<commit_message>
feat: Wave F real ingest path (disk fixtures, upload API, multi-employee)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/demo/smoke/peak_needs_ot/dec_demo_peak_ot_2026w40.xlsx
+++ b/artifacts/demo/smoke/peak_needs_ot/dec_demo_peak_ot_2026w40.xlsx
@@ -100,7 +100,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>sha256:f0c562e482ec3055d04a9e9701537362921e393dec7a5f0dff500ed8348660d2</t>
+          <t>sha256:8742cdc0edb082f05c08c5e2774d828c4551f9bbb3c19f8637f24df780b81bf8</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -177,12 +177,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>sha256:f0c562e482ec3055d04a9e9701537362921e393dec7a5f0dff500ed8348660d2</t>
+          <t>sha256:8742cdc0edb082f05c08c5e2774d828c4551f9bbb3c19f8637f24df780b81bf8</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>sam</t>
+          <t>jordan</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -254,12 +254,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sha256:f0c562e482ec3055d04a9e9701537362921e393dec7a5f0dff500ed8348660d2</t>
+          <t>sha256:8742cdc0edb082f05c08c5e2774d828c4551f9bbb3c19f8637f24df780b81bf8</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>sam</t>
+          <t>jordan</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -331,12 +331,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>sha256:f0c562e482ec3055d04a9e9701537362921e393dec7a5f0dff500ed8348660d2</t>
+          <t>sha256:8742cdc0edb082f05c08c5e2774d828c4551f9bbb3c19f8637f24df780b81bf8</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>sam</t>
+          <t>jordan</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -408,12 +408,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sha256:f0c562e482ec3055d04a9e9701537362921e393dec7a5f0dff500ed8348660d2</t>
+          <t>sha256:8742cdc0edb082f05c08c5e2774d828c4551f9bbb3c19f8637f24df780b81bf8</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sam</t>
+          <t>jordan</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>